<commit_message>
Updated Interfaces and N2 Diagram for WS2
</commit_message>
<xml_diff>
--- a/Explainer Demo/Physical Architecture Interfaces.xlsx
+++ b/Explainer Demo/Physical Architecture Interfaces.xlsx
@@ -20,9 +20,138 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t xml:space="preserve">TBD</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="44">
+  <si>
+    <t xml:space="preserve">Mechanical Interfaces N2 Diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whole System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whole Plane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airframe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuselage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propulsion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turbine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal Ducting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wing Control Surfaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tail Control Surfaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actuating Vents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Computing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ground</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transmitter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live Telemetry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“There in an interface from [left] to [top].” </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mechanical Interface:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“[left] is mounted to [top].”</t>
   </si>
 </sst>
 </file>
@@ -56,20 +185,137 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF666666"/>
+        <bgColor rgb="FF808080"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="16">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -98,8 +344,104 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -112,6 +454,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666666"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -292,15 +694,713 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:V24"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="3" style="0" width="5.71"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="C2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="V2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="13"/>
+      <c r="J6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="13"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="P6" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q6" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="R6" s="8"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" s="6"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="R7" s="8"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="17"/>
+      <c r="N8" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="O8" s="18"/>
+      <c r="P8" s="16"/>
+      <c r="Q8" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="R8" s="8"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
+      <c r="V9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="13"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="R10" s="8"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="15"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="6"/>
+      <c r="V11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="9"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
+      <c r="V12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="14"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="R13" s="8"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="14"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="14"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="R14" s="8"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
+      <c r="V14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="16"/>
+      <c r="Q15" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="R15" s="8"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="21"/>
+      <c r="Q16" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="R16" s="8"/>
+      <c r="S16" s="6"/>
+      <c r="T16" s="6"/>
+      <c r="U16" s="6"/>
+      <c r="V16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="20"/>
+      <c r="T17" s="20"/>
+      <c r="U17" s="20"/>
+      <c r="V17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="7"/>
+      <c r="V18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="6"/>
+      <c r="T19" s="6"/>
+      <c r="U19" s="6"/>
+      <c r="V19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="6"/>
+      <c r="T20" s="6"/>
+      <c r="U20" s="6"/>
+      <c r="V20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="8"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="6"/>
+      <c r="V21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2"/>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>43</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:U1"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>